<commit_message>
Weekly watchlist workbook — 2026-10-31 06:41 SAST
</commit_message>
<xml_diff>
--- a/reports/LRC_Watchlist_2026-10-23.xlsx
+++ b/reports/LRC_Watchlist_2026-10-23.xlsx
@@ -707,61 +707,61 @@
     <t xml:space="preserve">Trigger: Sell stop below the 15-day low (49.11) — only AFTER the 14 Oct results are digested. Short entry 49.00, stop 50.96 (2×ATR 0.98), target 43.12 (3R). LRC Work-sheet 14 Oct: SELL (6-m target ~$38.37, -25%; score 3.5/5; technical: CLEARED — STAGED ENTRY). SELL (−25%) + technical clearance. Results 14 Oct (today) — wait for the reaction. 5th short: house limit is 4 open shorts, so only if one of the others has not triggered. Data 13 Oct close: stockanalysis statistics + daily history to 13 Oct (SMA20/ATR14 computed); Perf Half vs ~13 Apr close; EPS growth this yr = consensus current FY (adjusted). Perf Quarter n/f (history page holds 50 sessions). Finviz itself blocked for us — same filters applied manually. — P. Nkuna</t>
   </si>
   <si>
+    <t xml:space="preserve">NVIDIA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LONG: Trend continuation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Agent 2026-10-25T15:09+02:00: LRC rating BUY (6-m value 262.56); NOT CLEARED. Entry 219.32, stop 207.2 (2×ATR), target 255.68 (3R).  — LRC Watchlist</t>
+  </si>
+  <si>
     <t xml:space="preserve">Intuit</t>
   </si>
   <si>
-    <t xml:space="preserve">LONG: Trend continuation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Agent 2026-10-24T06:26+02:00: LRC rating BUY (6-m value 426.0); NOT CLEARED. Entry 358.75, stop 332.97 (2×ATR), target 436.09 (3R).  — LRC Watchlist Agent</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NVIDIA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Agent 2026-10-24T06:26+02:00: LRC rating BUY (6-m value 262.56); NOT CLEARED. Entry 219.32, stop 207.2 (2×ATR), target 255.68 (3R).  — LRC Watchlist Agent</t>
+    <t xml:space="preserve">Agent 2026-10-25T15:09+02:00: LRC rating BUY (6-m value 426.0); NOT CLEARED. Entry 358.75, stop 332.97 (2×ATR), target 436.09 (3R).  — LRC Watchlist</t>
   </si>
   <si>
     <t xml:space="preserve">Deckers Outdoor</t>
   </si>
   <si>
-    <t xml:space="preserve">Agent 2026-10-24T06:26+02:00: LRC rating BUY (6-m value 103.0); NOT CLEARED. Entry 88.1, stop 82.28 (2×ATR), target 105.56 (3R).  — LRC Watchlist Agent</t>
+    <t xml:space="preserve">Agent 2026-10-25T15:09+02:00: LRC rating BUY (6-m value 103.0); NOT CLEARED. Entry 88.1, stop 82.28 (2×ATR), target 105.56 (3R).  — LRC Watchlist</t>
   </si>
   <si>
     <t xml:space="preserve">Wabtec</t>
   </si>
   <si>
-    <t xml:space="preserve">Agent 2026-10-24T06:26+02:00: LRC rating SELL (6-m value 248.07); CLEARED. Entry 270.6, stop 285.66 (2×ATR), target 225.42 (3R).  — LRC Watchlist Agent</t>
+    <t xml:space="preserve">Agent 2026-10-25T15:09+02:00: LRC rating SELL (6-m value 248.07); CLEARED. Entry 270.6, stop 285.66 (2×ATR), target 225.42 (3R).  — LRC Watchlist</t>
   </si>
   <si>
     <t xml:space="preserve">Nike</t>
   </si>
   <si>
-    <t xml:space="preserve">Agent 2026-10-24T06:26+02:00: LRC rating SELL (6-m value 29.75); CLEARED. Entry 32.69, stop 34.87 (2×ATR), target 26.15 (3R).  — LRC Watchlist Agent</t>
+    <t xml:space="preserve">Agent 2026-10-25T15:09+02:00: LRC rating SELL (6-m value 29.75); CLEARED. Entry 32.69, stop 34.87 (2×ATR), target 26.15 (3R).  — LRC Watchlist</t>
   </si>
   <si>
     <t xml:space="preserve">Arista Networks</t>
   </si>
   <si>
-    <t xml:space="preserve">Agent 2026-10-24T06:26+02:00: LRC rating SELL (6-m value 144.61); CLEARED — results within 14 days. Entry 167.9, stop 185.06 (2×ATR), target 116.42 (3R). Results 2026-11-03 — LRC Watchlist Agent</t>
+    <t xml:space="preserve">Agent 2026-10-25T15:09+02:00: LRC rating SELL (6-m value 144.61); CLEARED — results within 14 days. Entry 167.9, stop 185.06 (2×ATR), target 116.42 (3R). Results 2026-11-03 — LRC Watchlist</t>
   </si>
   <si>
     <t xml:space="preserve">Dell Technologies</t>
   </si>
   <si>
-    <t xml:space="preserve">Agent 2026-10-24T06:26+02:00: LRC rating SELL (6-m value 404.7); CLEARED. Entry 438.62, stop 500.56 (2×ATR), target 252.8 (3R).  — LRC Watchlist Agent</t>
+    <t xml:space="preserve">Agent 2026-10-25T15:09+02:00: LRC rating SELL (6-m value 404.7); CLEARED. Entry 438.62, stop 500.56 (2×ATR), target 252.8 (3R).  — LRC Watchlist</t>
   </si>
   <si>
     <t xml:space="preserve">Advanced Micro Devices</t>
   </si>
   <si>
-    <t xml:space="preserve">Agent 2026-10-24T06:26+02:00: LRC rating SELL (6-m value 402.73); CLEARED — results within 14 days. Entry 501.59, stop 556.31 (2×ATR), target 337.43 (3R). Results 2026-11-03; house limit: max 4 shorts — LRC Watchlist Agent</t>
+    <t xml:space="preserve">Agent 2026-10-25T15:09+02:00: LRC rating SELL (6-m value 402.73); CLEARED — results within 14 days. Entry 501.59, stop 556.31 (2×ATR), target 337.43 (3R). Results 2026-11-03; house limit: max 4 shorts — LRC Watchlist</t>
   </si>
   <si>
     <t xml:space="preserve">Fastenal</t>
   </si>
   <si>
-    <t xml:space="preserve">Agent 2026-10-24T06:26+02:00: LRC rating SELL (6-m value 38.37); CLEARED. Entry 47.21, stop 49.87 (2×ATR), target 39.23 (3R). house limit: max 4 shorts — LRC Watchlist Agent</t>
+    <t xml:space="preserve">Agent 2026-10-25T15:09+02:00: LRC rating SELL (6-m value 38.37); CLEARED. Entry 47.21, stop 49.87 (2×ATR), target 39.23 (3R). house limit: max 4 shorts — LRC Watchlist</t>
   </si>
   <si>
     <t xml:space="preserve">Weekly Review — swing (every weekend)</t>
@@ -845,7 +845,7 @@
     <t xml:space="preserve">Finviz is blocked for our tools, so the Swing Long / Swing Short presets were applied manually on stockanalysis.com data (13 Oct closes). LRC RULE: only BUY/SELL-rated names with technical clearance are tradeable. LONGS: only NVDA qualifies; INTU and DECK are BUY-rated but in downtrends (watch only). 2 long slots unfilled — the momentum names the long preset finds (DELL, HPE, KEYS, APH, AMD) all rate SELL on valuation. SHORTS: NKE, ANET, AMD, DELL, FAST (max 4 open; FAST only after its 14 Oct results). Event risk inside 14 days: WAB 21 Oct, DECK 22 Oct, META 21 Oct, APH/GOOGL 28 Oct. S&amp;P 500 above its 200-day; JSE All Share below (−7.4% in 6 months). Lesson: an un-entered trigger cost us the PCTY move (+9%) — set conditional orders when a setup is approved. — P. Nkuna</t>
   </si>
   <si>
-    <t xml:space="preserve">Built by the LRC Watchlist Agent 2026-10-24T06:26+02:00: 3 long / 6 short candidates under house rules. Analyst to review before any trade.</t>
+    <t xml:space="preserve">Built by the LRC Watchlist 2026-10-25T15:09+02:00: 3 long / 6 short candidates under house rules. Analyst to review before any trade.</t>
   </si>
   <si>
     <t xml:space="preserve">How to pick long-term investments (hold 5 to 10+ years) — every month</t>
@@ -2597,9 +2597,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>865440</xdr:colOff>
+      <xdr:colOff>865080</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>570240</xdr:rowOff>
+      <xdr:rowOff>569880</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2613,7 +2613,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="865440" cy="570240"/>
+          <a:ext cx="865080" cy="569880"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2640,9 +2640,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>420840</xdr:colOff>
+      <xdr:colOff>420480</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>570240</xdr:rowOff>
+      <xdr:rowOff>569880</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2656,7 +2656,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="865440" cy="570240"/>
+          <a:ext cx="865080" cy="569880"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2683,9 +2683,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>865440</xdr:colOff>
+      <xdr:colOff>865080</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>570240</xdr:rowOff>
+      <xdr:rowOff>569880</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2699,7 +2699,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="865440" cy="570240"/>
+          <a:ext cx="865080" cy="569880"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2726,9 +2726,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>865440</xdr:colOff>
+      <xdr:colOff>865080</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>570240</xdr:rowOff>
+      <xdr:rowOff>569880</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2742,7 +2742,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="865440" cy="570240"/>
+          <a:ext cx="865080" cy="569880"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2769,9 +2769,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>865440</xdr:colOff>
+      <xdr:colOff>865080</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>570240</xdr:rowOff>
+      <xdr:rowOff>569880</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2785,7 +2785,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="865440" cy="570240"/>
+          <a:ext cx="865080" cy="569880"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2812,9 +2812,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>865440</xdr:colOff>
+      <xdr:colOff>865080</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>570240</xdr:rowOff>
+      <xdr:rowOff>569880</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2828,7 +2828,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="865440" cy="570240"/>
+          <a:ext cx="865080" cy="569880"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2855,9 +2855,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>865440</xdr:colOff>
+      <xdr:colOff>865080</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>570240</xdr:rowOff>
+      <xdr:rowOff>569880</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2871,7 +2871,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="865440" cy="570240"/>
+          <a:ext cx="865080" cy="569880"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2898,9 +2898,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>865440</xdr:colOff>
+      <xdr:colOff>865080</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>570240</xdr:rowOff>
+      <xdr:rowOff>569880</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2914,7 +2914,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="865440" cy="570240"/>
+          <a:ext cx="865080" cy="569880"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2941,9 +2941,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>865440</xdr:colOff>
+      <xdr:colOff>865080</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>570240</xdr:rowOff>
+      <xdr:rowOff>569880</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2957,7 +2957,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="865440" cy="570240"/>
+          <a:ext cx="865080" cy="569880"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -4021,15 +4021,15 @@
       </c>
       <c r="B18" s="14" t="str">
         <f aca="false">IFERROR(INDEX('Swing Watchlist'!$C$11:$C$210,MATCH(LARGE('Swing Watchlist'!$AX$11:$AX$210,3),'Swing Watchlist'!$AX$11:$AX$210,0)),"")</f>
-        <v>DELL</v>
+        <v>NVDA</v>
       </c>
       <c r="C18" s="15" t="str">
         <f aca="false">IFERROR(IF(INDEX('Swing Watchlist'!$F$11:$F$210,MATCH(LARGE('Swing Watchlist'!$AX$11:$AX$210,3),'Swing Watchlist'!$AX$11:$AX$210,0))="Short","Short","Long"),"")</f>
-        <v>Short</v>
+        <v>Long</v>
       </c>
       <c r="D18" s="16" t="n">
         <f aca="false">IFERROR(INDEX('Swing Watchlist'!$AJ$11:$AJ$210,MATCH(LARGE('Swing Watchlist'!$AX$11:$AX$210,3),'Swing Watchlist'!$AX$11:$AX$210,0)),"")</f>
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E18" s="15" t="str">
         <f aca="false">IFERROR(INDEX('Swing Watchlist'!$AK$11:$AK$210,MATCH(LARGE('Swing Watchlist'!$AX$11:$AX$210,3),'Swing Watchlist'!$AX$11:$AX$210,0)),"")</f>
@@ -4070,7 +4070,7 @@
       </c>
       <c r="B19" s="14" t="str">
         <f aca="false">IFERROR(INDEX('Swing Watchlist'!$C$11:$C$210,MATCH(LARGE('Swing Watchlist'!$AX$11:$AX$210,4),'Swing Watchlist'!$AX$11:$AX$210,0)),"")</f>
-        <v>ANET</v>
+        <v>DELL</v>
       </c>
       <c r="C19" s="15" t="str">
         <f aca="false">IFERROR(IF(INDEX('Swing Watchlist'!$F$11:$F$210,MATCH(LARGE('Swing Watchlist'!$AX$11:$AX$210,4),'Swing Watchlist'!$AX$11:$AX$210,0))="Short","Short","Long"),"")</f>
@@ -4119,11 +4119,11 @@
       </c>
       <c r="B20" s="14" t="str">
         <f aca="false">IFERROR(INDEX('Swing Watchlist'!$C$11:$C$210,MATCH(LARGE('Swing Watchlist'!$AX$11:$AX$210,5),'Swing Watchlist'!$AX$11:$AX$210,0)),"")</f>
-        <v>NVDA</v>
+        <v>ANET</v>
       </c>
       <c r="C20" s="15" t="str">
         <f aca="false">IFERROR(IF(INDEX('Swing Watchlist'!$F$11:$F$210,MATCH(LARGE('Swing Watchlist'!$AX$11:$AX$210,5),'Swing Watchlist'!$AX$11:$AX$210,0))="Short","Short","Long"),"")</f>
-        <v>Long</v>
+        <v>Short</v>
       </c>
       <c r="D20" s="16" t="n">
         <f aca="false">IFERROR(INDEX('Swing Watchlist'!$AJ$11:$AJ$210,MATCH(LARGE('Swing Watchlist'!$AX$11:$AX$210,5),'Swing Watchlist'!$AX$11:$AX$210,0)),"")</f>
@@ -7091,7 +7091,7 @@
         <v>179</v>
       </c>
       <c r="C22" s="35" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="D22" s="35" t="s">
         <v>224</v>
@@ -7103,66 +7103,68 @@
         <v>183</v>
       </c>
       <c r="G22" s="26" t="n">
-        <v>343.39</v>
-      </c>
-      <c r="H22" s="26"/>
+        <v>210.96</v>
+      </c>
+      <c r="H22" s="26" t="n">
+        <v>5090</v>
+      </c>
       <c r="I22" s="36" t="n">
-        <v>3794424</v>
+        <v>116520944</v>
       </c>
       <c r="J22" s="37" t="n">
         <f aca="false">IF(OR(G22="",I22=""),"",G22*I22/1000000)</f>
-        <v>1302.96725736</v>
+        <v>24581.25834624</v>
       </c>
       <c r="K22" s="21" t="n">
-        <v>0.1216</v>
+        <v>-0.0646</v>
       </c>
       <c r="L22" s="21" t="n">
-        <v>0.0694</v>
+        <v>-0.0518</v>
       </c>
       <c r="M22" s="21" t="n">
-        <v>-0.0662</v>
+        <v>0.0358</v>
       </c>
       <c r="N22" s="25" t="n">
-        <v>64.05</v>
+        <v>38.09</v>
       </c>
       <c r="O22" s="21" t="n">
-        <v>0.1299</v>
+        <v>0.0735</v>
       </c>
       <c r="P22" s="21" t="n">
-        <v>-0.1327</v>
+        <v>0.0129</v>
       </c>
       <c r="Q22" s="21" t="n">
-        <v>-0.5017</v>
+        <v>-0.1332</v>
       </c>
       <c r="R22" s="21" t="n">
-        <v>0.3581</v>
+        <v>0.2842</v>
       </c>
       <c r="S22" s="38" t="n">
-        <v>0.67</v>
+        <v>0.69</v>
       </c>
       <c r="T22" s="21" t="n">
-        <v>-0.0133</v>
+        <v>0.9523</v>
       </c>
       <c r="U22" s="21" t="n">
-        <v>0.0279</v>
+        <v>0.0134</v>
       </c>
       <c r="V22" s="19" t="n">
-        <v>46345</v>
+        <v>46344</v>
       </c>
       <c r="W22" s="26" t="n">
-        <v>12.89</v>
+        <v>6.06</v>
       </c>
       <c r="X22" s="35" t="s">
         <v>225</v>
       </c>
       <c r="Y22" s="26" t="n">
-        <v>358.75</v>
+        <v>219.32</v>
       </c>
       <c r="Z22" s="26" t="n">
-        <v>332.97</v>
+        <v>207.2</v>
       </c>
       <c r="AA22" s="26" t="n">
-        <v>436.09</v>
+        <v>255.68</v>
       </c>
       <c r="AB22" s="16" t="n">
         <f aca="false">IF(C22="","",IF(F22="Short",(AND(M22&lt;&gt;"",N(M22)&lt;0))+(AND(L22&lt;&gt;"",N(L22)&lt;0))+(AND(K22&lt;&gt;"",N(K22)&lt;0))+AND(L22&lt;&gt;"",M22&lt;&gt;"",N(M22)&lt;N(L22)),(N(M22)&gt;0)+(N(L22)&gt;0)+(N(K22)&gt;0)+AND(L22&lt;&gt;"",M22&lt;&gt;"",N(M22)&gt;N(L22))))</f>
@@ -7170,11 +7172,11 @@
       </c>
       <c r="AC22" s="16" t="n">
         <f aca="false">IF(C22="","",IF(F22="Short",IF(N22="",0,IF(AND(N22&gt;=30,N22&lt;=50),2,IF(OR(AND(N22&gt;=25,N22&lt;30),AND(N22&gt;50,N22&lt;=60)),1,0)))+IF(P22="",0,IF(AND(IF(B22="JSE",$L$5,$L$4)&lt;&gt;"",P22&lt;IF(B22="JSE",$L$5,$L$4)),2,IF(P22&lt;0,1,0))),IF(N22="",0,IF(AND(N22&gt;=50,N22&lt;=70),2,IF(OR(AND(N22&gt;=40,N22&lt;50),AND(N22&gt;70,N22&lt;=75)),1,0)))+IF(P22="",0,IF(AND(IF(B22="JSE",$L$5,$L$4)&lt;&gt;"",P22&gt;IF(B22="JSE",$L$5,$L$4)),2,IF(P22&gt;0,1,0)))))</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AD22" s="16" t="n">
         <f aca="false">IF(C22="","",IF(F22="Short",IF(R22="",0,IF(R22&lt;=0.1,2,IF(R22&lt;=0.25,1,0))),IF(Q22="",0,IF(Q22&gt;=-0.1,2,IF(Q22&gt;=-0.25,1,0)))))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AE22" s="16" t="n">
         <f aca="false">IF(C22="","",IF(J22="",0,IF(J22&gt;=IF(B22="JSE",$L$7,$L$6),2,IF(J22&gt;=IF(B22="JSE",$L$7,$L$6)/4,1,0))))</f>
@@ -7182,7 +7184,7 @@
       </c>
       <c r="AF22" s="16" t="n">
         <f aca="false">IF(C22="","",IF(F22="Short",AND(T22&lt;&gt;"",N(T22)&lt;0),N(T22)&gt;0)+(N(S22)&gt;=1.5))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG22" s="16" t="n">
         <f aca="false">IF(C22="","",IF(AL22="",0,IF(AL22&gt;=3,4,IF(AL22&gt;=2,2,0))))</f>
@@ -7198,7 +7200,7 @@
       </c>
       <c r="AJ22" s="23" t="n">
         <f aca="false">IF(C22="","",SUM(AB22:AI22))</f>
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="AK22" s="24" t="str">
         <f aca="false">IF(C22="","",IF(AJ22&gt;=14,"A",IF(AJ22&gt;=10,"B","C")))</f>
@@ -7210,15 +7212,15 @@
       </c>
       <c r="AM22" s="37" t="n">
         <f aca="false">IF(OR(Y22="",Z22="",N(Y22)=N(Z22)),"",IF(OR(AND(F22="Short",Z22&lt;Y22),AND(NOT(F22="Short"),Z22&gt;Y22)),"stop on wrong side",ABS(Y22-Z22)))</f>
-        <v>25.78</v>
+        <v>12.12</v>
       </c>
       <c r="AN22" s="40" t="n">
         <f aca="false">IFERROR(IF(OR(NOT(ISNUMBER(AM22)),$C$6=""),"",ROUNDDOWN($C$6*$C$7/AM22,2)),"")</f>
-        <v>0.01</v>
+        <v>0.03</v>
       </c>
       <c r="AO22" s="37" t="n">
         <f aca="false">IFERROR(IF(AN22="","",AN22*Y22),"")</f>
-        <v>3.5875</v>
+        <v>6.5796</v>
       </c>
       <c r="AP22" s="35" t="s">
         <v>192</v>
@@ -7242,7 +7244,7 @@
       </c>
       <c r="AX22" s="43" t="n">
         <f aca="false">IF(AND(C22&lt;&gt;"",A22=$C$4,ISNUMBER(AJ22)),AJ22+ROW()/100000,"")</f>
-        <v>10.00022</v>
+        <v>11.00022</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7253,7 +7255,7 @@
         <v>179</v>
       </c>
       <c r="C23" s="35" t="s">
-        <v>197</v>
+        <v>201</v>
       </c>
       <c r="D23" s="35" t="s">
         <v>227</v>
@@ -7265,64 +7267,68 @@
         <v>183</v>
       </c>
       <c r="G23" s="26" t="n">
-        <v>210.96</v>
-      </c>
-      <c r="H23" s="26"/>
+        <v>343.39</v>
+      </c>
+      <c r="H23" s="26" t="n">
+        <v>91.77</v>
+      </c>
       <c r="I23" s="36" t="n">
-        <v>116520944</v>
+        <v>3794424</v>
       </c>
       <c r="J23" s="37" t="n">
         <f aca="false">IF(OR(G23="",I23=""),"",G23*I23/1000000)</f>
-        <v>24581.25834624</v>
+        <v>1302.96725736</v>
       </c>
       <c r="K23" s="21" t="n">
-        <v>-0.0646</v>
+        <v>0.1216</v>
       </c>
       <c r="L23" s="21" t="n">
-        <v>-0.0518</v>
+        <v>0.0694</v>
       </c>
       <c r="M23" s="21" t="n">
-        <v>0.0358</v>
+        <v>-0.0662</v>
       </c>
       <c r="N23" s="25" t="n">
-        <v>38.09</v>
+        <v>64.05</v>
       </c>
       <c r="O23" s="21" t="n">
-        <v>0.0735</v>
+        <v>0.1299</v>
       </c>
       <c r="P23" s="21" t="n">
-        <v>0.0129</v>
+        <v>-0.1327</v>
       </c>
       <c r="Q23" s="21" t="n">
-        <v>-0.1332</v>
+        <v>-0.5017</v>
       </c>
       <c r="R23" s="21" t="n">
-        <v>0.2842</v>
+        <v>0.3581</v>
       </c>
       <c r="S23" s="38" t="n">
-        <v>0.69</v>
-      </c>
-      <c r="T23" s="21"/>
+        <v>0.67</v>
+      </c>
+      <c r="T23" s="21" t="n">
+        <v>-0.0189</v>
+      </c>
       <c r="U23" s="21" t="n">
-        <v>0.0134</v>
+        <v>0.0279</v>
       </c>
       <c r="V23" s="19" t="n">
-        <v>46344</v>
+        <v>46345</v>
       </c>
       <c r="W23" s="26" t="n">
-        <v>6.06</v>
+        <v>12.89</v>
       </c>
       <c r="X23" s="35" t="s">
         <v>225</v>
       </c>
       <c r="Y23" s="26" t="n">
-        <v>219.32</v>
+        <v>358.75</v>
       </c>
       <c r="Z23" s="26" t="n">
-        <v>207.2</v>
+        <v>332.97</v>
       </c>
       <c r="AA23" s="26" t="n">
-        <v>255.68</v>
+        <v>436.09</v>
       </c>
       <c r="AB23" s="16" t="n">
         <f aca="false">IF(C23="","",IF(F23="Short",(AND(M23&lt;&gt;"",N(M23)&lt;0))+(AND(L23&lt;&gt;"",N(L23)&lt;0))+(AND(K23&lt;&gt;"",N(K23)&lt;0))+AND(L23&lt;&gt;"",M23&lt;&gt;"",N(M23)&lt;N(L23)),(N(M23)&gt;0)+(N(L23)&gt;0)+(N(K23)&gt;0)+AND(L23&lt;&gt;"",M23&lt;&gt;"",N(M23)&gt;N(L23))))</f>
@@ -7330,11 +7336,11 @@
       </c>
       <c r="AC23" s="16" t="n">
         <f aca="false">IF(C23="","",IF(F23="Short",IF(N23="",0,IF(AND(N23&gt;=30,N23&lt;=50),2,IF(OR(AND(N23&gt;=25,N23&lt;30),AND(N23&gt;50,N23&lt;=60)),1,0)))+IF(P23="",0,IF(AND(IF(B23="JSE",$L$5,$L$4)&lt;&gt;"",P23&lt;IF(B23="JSE",$L$5,$L$4)),2,IF(P23&lt;0,1,0))),IF(N23="",0,IF(AND(N23&gt;=50,N23&lt;=70),2,IF(OR(AND(N23&gt;=40,N23&lt;50),AND(N23&gt;70,N23&lt;=75)),1,0)))+IF(P23="",0,IF(AND(IF(B23="JSE",$L$5,$L$4)&lt;&gt;"",P23&gt;IF(B23="JSE",$L$5,$L$4)),2,IF(P23&gt;0,1,0)))))</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AD23" s="16" t="n">
         <f aca="false">IF(C23="","",IF(F23="Short",IF(R23="",0,IF(R23&lt;=0.1,2,IF(R23&lt;=0.25,1,0))),IF(Q23="",0,IF(Q23&gt;=-0.1,2,IF(Q23&gt;=-0.25,1,0)))))</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AE23" s="16" t="n">
         <f aca="false">IF(C23="","",IF(J23="",0,IF(J23&gt;=IF(B23="JSE",$L$7,$L$6),2,IF(J23&gt;=IF(B23="JSE",$L$7,$L$6)/4,1,0))))</f>
@@ -7370,15 +7376,15 @@
       </c>
       <c r="AM23" s="37" t="n">
         <f aca="false">IF(OR(Y23="",Z23="",N(Y23)=N(Z23)),"",IF(OR(AND(F23="Short",Z23&lt;Y23),AND(NOT(F23="Short"),Z23&gt;Y23)),"stop on wrong side",ABS(Y23-Z23)))</f>
-        <v>12.12</v>
+        <v>25.78</v>
       </c>
       <c r="AN23" s="40" t="n">
         <f aca="false">IFERROR(IF(OR(NOT(ISNUMBER(AM23)),$C$6=""),"",ROUNDDOWN($C$6*$C$7/AM23,2)),"")</f>
-        <v>0.03</v>
+        <v>0.01</v>
       </c>
       <c r="AO23" s="37" t="n">
         <f aca="false">IFERROR(IF(AN23="","",AN23*Y23),"")</f>
-        <v>6.5796</v>
+        <v>3.5875</v>
       </c>
       <c r="AP23" s="35" t="s">
         <v>192</v>
@@ -7419,7 +7425,7 @@
         <v>229</v>
       </c>
       <c r="E24" s="35" t="s">
-        <v>182</v>
+        <v>207</v>
       </c>
       <c r="F24" s="35" t="s">
         <v>183</v>
@@ -7427,7 +7433,9 @@
       <c r="G24" s="26" t="n">
         <v>81.09</v>
       </c>
-      <c r="H24" s="26"/>
+      <c r="H24" s="26" t="n">
+        <v>11.04</v>
+      </c>
       <c r="I24" s="36" t="n">
         <v>3058068</v>
       </c>
@@ -7462,13 +7470,13 @@
       <c r="S24" s="38" t="n">
         <v>3.04</v>
       </c>
-      <c r="T24" s="21"/>
+      <c r="T24" s="21" t="n">
+        <v>0.0733</v>
+      </c>
       <c r="U24" s="21" t="n">
         <v>0.0877</v>
       </c>
-      <c r="V24" s="19" t="n">
-        <v>46317</v>
-      </c>
+      <c r="V24" s="19"/>
       <c r="W24" s="26" t="n">
         <v>2.91</v>
       </c>
@@ -7502,7 +7510,7 @@
       </c>
       <c r="AF24" s="16" t="n">
         <f aca="false">IF(C24="","",IF(F24="Short",AND(T24&lt;&gt;"",N(T24)&lt;0),N(T24)&gt;0)+(N(S24)&gt;=1.5))</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AG24" s="16" t="n">
         <f aca="false">IF(C24="","",IF(AL24="",0,IF(AL24&gt;=3,4,IF(AL24&gt;=2,2,0))))</f>
@@ -7518,7 +7526,7 @@
       </c>
       <c r="AJ24" s="23" t="n">
         <f aca="false">IF(C24="","",SUM(AB24:AI24))</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AK24" s="24" t="str">
         <f aca="false">IF(C24="","",IF(AJ24&gt;=14,"A",IF(AJ24&gt;=10,"B","C")))</f>
@@ -7562,7 +7570,7 @@
       </c>
       <c r="AX24" s="43" t="n">
         <f aca="false">IF(AND(C24&lt;&gt;"",A24=$C$4,ISNUMBER(AJ24)),AJ24+ROW()/100000,"")</f>
-        <v>8.00024</v>
+        <v>9.00024</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7579,7 +7587,7 @@
         <v>231</v>
       </c>
       <c r="E25" s="35" t="s">
-        <v>182</v>
+        <v>189</v>
       </c>
       <c r="F25" s="35" t="s">
         <v>190</v>
@@ -7587,7 +7595,9 @@
       <c r="G25" s="26" t="n">
         <v>272.35</v>
       </c>
-      <c r="H25" s="26"/>
+      <c r="H25" s="26" t="n">
+        <v>45.7</v>
+      </c>
       <c r="I25" s="36" t="n">
         <v>906852</v>
       </c>
@@ -7622,13 +7632,13 @@
       <c r="S25" s="38" t="n">
         <v>1.71</v>
       </c>
-      <c r="T25" s="21"/>
+      <c r="T25" s="21" t="n">
+        <v>0.2118</v>
+      </c>
       <c r="U25" s="21" t="n">
         <v>0.0212</v>
       </c>
-      <c r="V25" s="19" t="n">
-        <v>46316</v>
-      </c>
+      <c r="V25" s="19"/>
       <c r="W25" s="26" t="n">
         <v>7.53</v>
       </c>
@@ -7739,7 +7749,7 @@
         <v>233</v>
       </c>
       <c r="E26" s="35" t="s">
-        <v>182</v>
+        <v>207</v>
       </c>
       <c r="F26" s="35" t="s">
         <v>190</v>
@@ -7747,7 +7757,9 @@
       <c r="G26" s="26" t="n">
         <v>37.3</v>
       </c>
-      <c r="H26" s="26"/>
+      <c r="H26" s="26" t="n">
+        <v>55.4</v>
+      </c>
       <c r="I26" s="36" t="n">
         <v>33320533</v>
       </c>
@@ -7783,7 +7795,7 @@
         <v>0.78</v>
       </c>
       <c r="T26" s="21" t="n">
-        <v>-0.1642</v>
+        <v>-0.173</v>
       </c>
       <c r="U26" s="21" t="n">
         <v>0.0842</v>
@@ -7907,7 +7919,9 @@
       <c r="G27" s="26" t="n">
         <v>172.37</v>
       </c>
-      <c r="H27" s="26"/>
+      <c r="H27" s="26" t="n">
+        <v>217.4</v>
+      </c>
       <c r="I27" s="36" t="n">
         <v>6149214</v>
       </c>
@@ -7942,7 +7956,9 @@
       <c r="S27" s="38" t="n">
         <v>0.81</v>
       </c>
-      <c r="T27" s="21"/>
+      <c r="T27" s="21" t="n">
+        <v>0.3815</v>
+      </c>
       <c r="U27" s="21" t="n">
         <v>0.0114</v>
       </c>
@@ -8067,7 +8083,9 @@
       <c r="G28" s="26" t="n">
         <v>456.44</v>
       </c>
-      <c r="H28" s="26"/>
+      <c r="H28" s="26" t="n">
+        <v>290.21</v>
+      </c>
       <c r="I28" s="36" t="n">
         <v>7702417</v>
       </c>
@@ -8103,10 +8121,10 @@
         <v>0.56</v>
       </c>
       <c r="T28" s="21" t="n">
-        <v>1.514</v>
+        <v>1.5142</v>
       </c>
       <c r="U28" s="21" t="n">
-        <v>0.0469</v>
+        <v>0.0421</v>
       </c>
       <c r="V28" s="19" t="n">
         <v>46350</v>
@@ -8229,7 +8247,9 @@
       <c r="G29" s="26" t="n">
         <v>516.79</v>
       </c>
-      <c r="H29" s="26"/>
+      <c r="H29" s="26" t="n">
+        <v>843.65</v>
+      </c>
       <c r="I29" s="36" t="n">
         <v>22028486</v>
       </c>
@@ -8265,7 +8285,7 @@
         <v>0.69</v>
       </c>
       <c r="T29" s="21" t="n">
-        <v>0.819</v>
+        <v>0.8194</v>
       </c>
       <c r="U29" s="21" t="n">
         <v>0.0242</v>
@@ -8383,7 +8403,7 @@
         <v>241</v>
       </c>
       <c r="E30" s="35" t="s">
-        <v>182</v>
+        <v>189</v>
       </c>
       <c r="F30" s="35" t="s">
         <v>190</v>
@@ -8391,7 +8411,9 @@
       <c r="G30" s="26" t="n">
         <v>51.91</v>
       </c>
-      <c r="H30" s="26"/>
+      <c r="H30" s="26" t="n">
+        <v>59.56</v>
+      </c>
       <c r="I30" s="36" t="n">
         <v>7530214</v>
       </c>
@@ -8426,13 +8448,13 @@
       <c r="S30" s="38" t="n">
         <v>0.75</v>
       </c>
-      <c r="T30" s="21"/>
+      <c r="T30" s="21" t="n">
+        <v>0.1666</v>
+      </c>
       <c r="U30" s="21" t="n">
         <v>0.0302</v>
       </c>
-      <c r="V30" s="19" t="n">
-        <v>46309</v>
-      </c>
+      <c r="V30" s="19"/>
       <c r="W30" s="26" t="n">
         <v>1.33</v>
       </c>

</xml_diff>